<commit_message>
correcciones en carga masiva de productos
</commit_message>
<xml_diff>
--- a/src/assets/plantilla-listalo.xlsx
+++ b/src/assets/plantilla-listalo.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\facub\OneDrive\Documents\DesarrolloWeb\ProyectoCatalogo\ProyectoCatalogo-front\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA65FA42-3281-4EA3-8A72-FA1CB7C5CE0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8334C8A1-906F-4D8B-89DD-CEA8A8CF83A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="2790" windowWidth="21600" windowHeight="11295" xr2:uid="{B18C3C7B-2DB4-4E4C-A8AC-F28B3A563A95}"/>
+    <workbookView xWindow="3075" yWindow="2460" windowWidth="21600" windowHeight="11295" xr2:uid="{B18C3C7B-2DB4-4E4C-A8AC-F28B3A563A95}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Plantilla" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -81,18 +81,24 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4F46E5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -151,27 +157,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF4F46E5"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -503,42 +526,44 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="45.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="22" style="2" customWidth="1"/>
-    <col min="5" max="5" width="20" style="2" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="27.28515625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="32" style="2" customWidth="1"/>
+    <col min="2" max="2" width="48.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="22.5703125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="20" style="3" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="57.7109375" style="3" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F2" s="7"/>
+      <c r="F2" s="4"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="HQWSAYFySdNBKopqcUOxBNXumFNciJaZg5eZvcjvtuHOTa5h1GEGTMKfgUCuhyWGUHPSegR0zPVL54dYIGze3g==" saltValue="LQDlE8wIBq5zRb8SSeueTw==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
plantilla excel sin bloquearse
</commit_message>
<xml_diff>
--- a/src/assets/plantilla-listalo.xlsx
+++ b/src/assets/plantilla-listalo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\facub\OneDrive\Documents\DesarrolloWeb\ProyectoCatalogo\ProyectoCatalogo-front\src\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\facub\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8334C8A1-906F-4D8B-89DD-CEA8A8CF83A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E698D99A-D36B-470B-98F7-C5FBA64873D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="2460" windowWidth="21600" windowHeight="11295" xr2:uid="{B18C3C7B-2DB4-4E4C-A8AC-F28B3A563A95}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B18C3C7B-2DB4-4E4C-A8AC-F28B3A563A95}"/>
   </bookViews>
   <sheets>
     <sheet name="Plantilla" sheetId="1" r:id="rId1"/>
@@ -157,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -174,16 +174,15 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,7 +535,7 @@
     <col min="8" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>2</v>
       </c>
@@ -563,7 +562,7 @@
       <c r="F2" s="4"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="HQWSAYFySdNBKopqcUOxBNXumFNciJaZg5eZvcjvtuHOTa5h1GEGTMKfgUCuhyWGUHPSegR0zPVL54dYIGze3g==" saltValue="LQDlE8wIBq5zRb8SSeueTw==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>